<commit_message>
feat(migration): preview (dry run) and execute with file-hash guard
Sheet 7 is optional (a koperasi may have no loans). withManagedIdentity
accepts transaction options so bulk work is not cut off at 5s.

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/migration/SISKOP-Template-Migrasi-Laporan.xlsx
+++ b/docs/migration/SISKOP-Template-Migrasi-Laporan.xlsx
@@ -201,7 +201,7 @@
     <t>7_Pinjaman</t>
   </si>
   <si>
-    <t>WAJIB. Sisa pembiayaan per anggota dari lampiran RAT. Laporan tidak memuat plafon, tenor, atau tanggal cair, jadi sistem membuat nilai pengganti dan menandainya di Catatan. KOL dan jatuh tempo TIDAK akurat sampai kontrak asli dimasukkan.</t>
+    <t>opsional. Sisa pembiayaan per anggota dari lampiran RAT. Laporan tidak memuat plafon, tenor, atau tanggal cair, jadi sistem membuat nilai pengganti dan menandainya di Catatan. KOL dan jatuh tempo TIDAK akurat sampai kontrak asli dimasukkan. Kosongkan sheet ini bila koperasi belum punya pinjaman.</t>
   </si>
   <si>
     <t>9_Neraca</t>
@@ -45749,7 +45749,7 @@
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <sheetPr>
-    <tabColor rgb="FF1F3A5F"/>
+    <tabColor rgb="FF6B7280"/>
   </sheetPr>
   <dimension ref="A1:J1003"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>

</xml_diff>